<commit_message>
HOA budget template: corrected spreadsheet + page copy to match it
Client sent a corrected workbook (the prior one had errors) and revised page copy
so the guide and the template tell the same story.

- Replace public/downloads/cmgt-hoa-budget-template.xlsx with the corrected file.
- Rewrite the guide copy to match the workbook: the download describes the real
  tabs (Budget / optional Reserves / optional Cash Check / Example); the worked
  example is the Magnolia Bend Example tab line-by-line ($174.57 billed); income
  excludes assessments (dues come out of the math); step 5, the two FAQ answers,
  and the HowTo/FAQ JSON-LD updated to match; capital double-charge and the
  increase-cap added to the mistakes list; longer disclaimer; #free-template
  anchor; read time 9 min.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/cmgt-hoa-budget-template.xlsx
+++ b/public/downloads/cmgt-hoa-budget-template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="249">
   <si>
     <t xml:space="preserve">HOA Budget Template</t>
   </si>
@@ -128,10 +128,10 @@
     <t xml:space="preserve">You never type in assessment income. It's whatever the budget requires after other income, which is the only figure that actually balances.</t>
   </si>
   <si>
-    <t xml:space="preserve">Late payers never raise dues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dues are budgeted at 100% of the homes that pay. Collection risk is shown separately, so owners who pay on time aren't billed extra to cover those who don't.</t>
+    <t xml:space="preserve">Your cap is checked for you</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The increase is compared against the cap in your governing documents, with a three-year phase-in if the full increase isn't adoptable this year.</t>
   </si>
   <si>
     <t xml:space="preserve">Capital is charged once</t>
@@ -164,7 +164,7 @@
     <t xml:space="preserve">Step 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Read section 5: the required assessment and the change from today. Check it against your cap.</t>
+    <t xml:space="preserve">Read section 5: the billed assessment, grossed up for your delinquency allowance, and the change from today. Check it against your cap.</t>
   </si>
   <si>
     <t xml:space="preserve">Step 5</t>
@@ -245,10 +245,10 @@
     <t xml:space="preserve">Commonly 3% to 5%, for ordinary surprises, not storms or capital work.</t>
   </si>
   <si>
-    <t xml:space="preserve">Current delinquency rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only used to show collection exposure below. It never raises anyone's dues.</t>
+    <t xml:space="preserve">Delinquency allowance (share of dues you expect to arrive late)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bills are grossed up by this share so the plan still works when a few homeowners pay late. Base it on your community's history.</t>
   </si>
   <si>
     <t xml:space="preserve">2 · INCOME OTHER THAN ASSESSMENTS</t>
@@ -464,16 +464,22 @@
     <t xml:space="preserve">Assessment revenue required</t>
   </si>
   <si>
-    <t xml:space="preserve">Budgeted at 100% of the homes that pay. This is the only figure that balances the budget.</t>
+    <t xml:space="preserve">What dues need to bring in after other income.</t>
   </si>
   <si>
     <t xml:space="preserve">Required — per home, per year</t>
   </si>
   <si>
-    <t xml:space="preserve">REQUIRED — PER HOME, PER PAYMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What each homeowner would be billed each payment period.</t>
+    <t xml:space="preserve">Required — per home, per payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before the delinquency allowance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BILLED — PER HOME, PER PAYMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grossed up for the delinquency allowance. This is what each homeowner is billed.</t>
   </si>
   <si>
     <t xml:space="preserve">Change from current assessment — per payment</t>
@@ -512,27 +518,6 @@
     <t xml:space="preserve">Year 3</t>
   </si>
   <si>
-    <t xml:space="preserve">7 · COLLECTION EXPOSURE — SHOWN, NOT BUILT IN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assessment dollars at risk this year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Required assessments × your current delinquency rate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covered by contingency and operating cash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Your first line of defense against a collection gap.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uncovered exposure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dues are not raised to cover this. That would make the owners who pay subsidize the ones who don't. If this number is large, fix collections.</t>
-  </si>
-  <si>
     <t xml:space="preserve">A free planning tool from CMGT, not the process CMGT uses to prepare budgets for the communities it manages. Not accounting, tax, legal or financial advice; work with your CPA and your association's attorney. Adoption, notice and ratification rules vary by governing documents and state law. cmgt.org/resources/hoa-budget-template</t>
   </si>
   <si>
@@ -653,7 +638,7 @@
     <t xml:space="preserve">CASH IN</t>
   </si>
   <si>
-    <t xml:space="preserve">Assessments</t>
+    <t xml:space="preserve">Assessments (expected collections)</t>
   </si>
   <si>
     <t xml:space="preserve">By payment schedule</t>
@@ -1638,7 +1623,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
         <v>45</v>
       </c>
@@ -1690,7 +1675,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1831,7 +1816,7 @@
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
         <v>73</v>
       </c>
@@ -2396,11 +2381,10 @@
       <c r="E58" s="8"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="30" t="s">
+      <c r="A59" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="B59" s="31"/>
-      <c r="C59" s="32" t="str">
+      <c r="C59" s="29" t="str">
         <f aca="false">IF(OR($B$8=0,$B$9=0),"",C57/$B$8/$B$9)</f>
         <v/>
       </c>
@@ -2409,36 +2393,37 @@
       </c>
       <c r="E59" s="8"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="9" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="C60" s="29" t="str">
-        <f aca="false">IF(OR(C59="",$B$10=0),"",C59-$B$10)</f>
-        <v/>
-      </c>
-      <c r="D60" s="8"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="32" t="str">
+        <f aca="false">IF(C59="","",C59/(1-$B$14))</f>
+        <v/>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>151</v>
+      </c>
       <c r="E60" s="8"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="C61" s="33" t="str">
-        <f aca="false">IF(OR(C59="",$B$10=0),"",C59/$B$10-1)</f>
-        <v/>
-      </c>
-      <c r="D61" s="8" t="s">
         <v>152</v>
       </c>
+      <c r="C61" s="29" t="str">
+        <f aca="false">IF(OR(C60="",$B$10=0),"",C60-$B$10)</f>
+        <v/>
+      </c>
+      <c r="D61" s="8"/>
       <c r="E61" s="8"/>
     </row>
-    <row r="62" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="C62" s="24" t="str">
-        <f aca="false">IF(C61="","",IF($B$12="","No cap entered",IF(C61&lt;=$B$12,"Yes","Over the cap — check your documents")))</f>
+      <c r="C62" s="33" t="str">
+        <f aca="false">IF(OR(C60="",$B$10=0),"",C60/$B$10-1)</f>
         <v/>
       </c>
       <c r="D62" s="8" t="s">
@@ -2446,132 +2431,97 @@
       </c>
       <c r="E62" s="8"/>
     </row>
-    <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="25" t="s">
+    <row r="63" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="B64" s="26"/>
-      <c r="C64" s="26"/>
-      <c r="D64" s="26"/>
-      <c r="E64" s="26"/>
-    </row>
-    <row r="65" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="8" t="s">
+      <c r="C63" s="24" t="str">
+        <f aca="false">IF(C62="","",IF($B$12="","No cap entered",IF(C62&lt;=$B$12,"Yes","Over the cap — check your documents")))</f>
+        <v/>
+      </c>
+      <c r="D63" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="B65" s="8"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="8"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="34"/>
-      <c r="B66" s="35" t="s">
+      <c r="E63" s="8"/>
+    </row>
+    <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="C66" s="35" t="s">
+      <c r="B65" s="26"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="26"/>
+    </row>
+    <row r="66" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="8" t="s">
         <v>158</v>
       </c>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="24" t="s">
+      <c r="A67" s="34"/>
+      <c r="B67" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="B67" s="29" t="str">
-        <f aca="false">IF(C$59="","",IF($B$12="",C$59,MIN(C$59,$B$10*(1+$B$12))))</f>
-        <v/>
-      </c>
-      <c r="C67" s="17" t="str">
-        <f aca="false">IF(B67="","",(C$59-B67)*$B$8*$B$9)</f>
-        <v/>
+      <c r="C67" s="35" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B68" s="29" t="str">
-        <f aca="false">IF(C$59="","",IF($B$12="",C$59,MIN(C$59,B67*(1+$B$12))))</f>
+        <f aca="false">IF(C$60="","",IF($B$12="",C$60,MIN(C$60,$B$10*(1+$B$12))))</f>
         <v/>
       </c>
       <c r="C68" s="17" t="str">
-        <f aca="false">IF(B68="","",(C$59-B68)*$B$8*$B$9)</f>
+        <f aca="false">IF(B68="","",(C$60-B68)*$B$8*$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B69" s="29" t="str">
-        <f aca="false">IF(C$59="","",IF($B$12="",C$59,MIN(C$59,B68*(1+$B$12))))</f>
+        <f aca="false">IF(C$60="","",IF($B$12="",C$60,MIN(C$60,B68*(1+$B$12))))</f>
         <v/>
       </c>
       <c r="C69" s="17" t="str">
-        <f aca="false">IF(B69="","",(C$59-B69)*$B$8*$B$9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="26"/>
-      <c r="E71" s="26"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="9" t="s">
+        <f aca="false">IF(B69="","",(C$60-B69)*$B$8*$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="C72" s="17" t="n">
-        <f aca="false">C57*$B$14</f>
-        <v>0</v>
-      </c>
-      <c r="D72" s="8" t="s">
+      <c r="B70" s="29" t="str">
+        <f aca="false">IF(C$60="","",IF($B$12="",C$60,MIN(C$60,B69*(1+$B$12))))</f>
+        <v/>
+      </c>
+      <c r="C70" s="17" t="str">
+        <f aca="false">IF(B70="","",(C$60-B70)*$B$8*$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="8" t="s">
         <v>164</v>
       </c>
+      <c r="B72" s="8"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="8"/>
       <c r="E72" s="8"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="C73" s="17" t="n">
-        <f aca="false">C50+$B$11</f>
-        <v>0</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="E73" s="8"/>
-    </row>
-    <row r="74" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="C74" s="17" t="n">
-        <f aca="false">MAX(0,C72-C73)</f>
-        <v>0</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="E74" s="8"/>
-    </row>
-    <row r="76" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
     </row>
   </sheetData>
   <sheetProtection sheet="true" formatColumns="false" formatRows="false"/>
-  <mergeCells count="25">
+  <mergeCells count="23">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="C5:E5"/>
@@ -2592,11 +2542,9 @@
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="D61:E61"/>
     <mergeCell ref="D62:E62"/>
-    <mergeCell ref="A65:E65"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A72:E72"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B9" type="list">
@@ -2647,7 +2595,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2658,7 +2606,7 @@
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -2669,25 +2617,25 @@
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="G5" s="16" t="s">
         <v>173</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2872,7 +2820,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -2883,7 +2831,7 @@
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -2894,11 +2842,11 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="24" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
@@ -2906,14 +2854,14 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="24" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C22" s="17" t="n">
         <f aca="false">SUM(F6:F17)</f>
         <v>0</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
@@ -2921,14 +2869,14 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="24" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C23" s="33" t="str">
         <f aca="false">IF(C22=0,"",C21/C22)</f>
         <v/>
       </c>
       <c r="D23" s="8" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
@@ -2936,13 +2884,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="24" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C24" s="36" t="n">
         <v>10</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -2950,14 +2898,14 @@
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C25" s="20" t="n">
         <f aca="false">SUM(E6:E17)+IF(C24=0,0,MAX(0,C22-C21)/C24)</f>
         <v>0</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
@@ -2965,7 +2913,7 @@
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2976,16 +2924,16 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3080,12 +3028,12 @@
     </row>
     <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="21" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="19" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C42" s="20" t="n">
         <f aca="false">SUM(E30:E39)</f>
@@ -3094,7 +3042,7 @@
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -3167,7 +3115,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3186,13 +3134,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="24" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B4" s="11" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
@@ -3209,7 +3157,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>3</v>
@@ -3230,7 +3178,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>6</v>
@@ -3252,10 +3200,10 @@
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37"/>
       <c r="B8" s="19" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D8" s="38" t="str">
         <f aca="false">CHOOSE(D9,"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec")</f>
@@ -3306,12 +3254,12 @@
         <v>Dec</v>
       </c>
       <c r="Q8" s="34" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D9" s="39" t="n">
         <f aca="false">MOD(Budget!$B$7-1+0,12)+1</f>
@@ -3364,7 +3312,7 @@
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -3383,14 +3331,14 @@
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">Budget!$C$57</f>
         <v>0</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="D11" s="17" t="n">
         <f aca="false">IF(OR(Budget!$B$9=0,MOD((COLUMN()-3)-1,12/Budget!$B$9)&lt;&gt;0),0,$B11/Budget!$B$9)</f>
@@ -3454,7 +3402,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D12" s="17" t="n">
         <f aca="false">$B12/12</f>
@@ -3511,7 +3459,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B13" s="20" t="n">
         <f aca="false">SUM(B11:B12)</f>
@@ -3569,7 +3517,7 @@
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -3588,14 +3536,14 @@
     </row>
     <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">(Budget!$C$27+Budget!$C$28+Budget!$C$29+Budget!$C$30)</f>
         <v>0</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D16" s="17" t="n">
         <f aca="false">IF(D$9=$B$4,$B16,0)</f>
@@ -3652,14 +3600,14 @@
     </row>
     <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="24" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">(Budget!$C$39+Budget!$C$41)</f>
         <v>0</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="D17" s="17" t="n">
         <f aca="false">IF(D$9=$B$5,$B17,0)</f>
@@ -3723,7 +3671,7 @@
         <v>0</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="D18" s="17" t="n">
         <f aca="false">IF(AND(D$9&gt;=5,D$9&lt;=9),$B18/5,0)</f>
@@ -3780,14 +3728,14 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="24" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">Budget!$C$44-(Budget!$C$27+Budget!$C$28+Budget!$C$29+Budget!$C$30)-(Budget!$C$39+Budget!$C$41)-Budget!$C$35</f>
         <v>0</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D19" s="17" t="n">
         <f aca="false">$B19/12</f>
@@ -3844,14 +3792,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="24" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">Budget!$C$47+Budget!$C$49+Budget!$C$50</f>
         <v>0</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D20" s="17" t="n">
         <f aca="false">$B20/12</f>
@@ -3908,14 +3856,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="24" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">Budget!$C$51</f>
         <v>0</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="D21" s="17" t="n">
         <f aca="false">IF(D$9=$B$6,$B21,0)</f>
@@ -3972,7 +3920,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B22" s="20" t="n">
         <f aca="false">SUM(B16:B21)</f>
@@ -4030,7 +3978,7 @@
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -4049,7 +3997,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="24" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="D25" s="22" t="n">
         <f aca="false">Budget!$B$11</f>
@@ -4102,7 +4050,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D26" s="20" t="n">
         <f aca="false">D25+D13-D22</f>
@@ -4155,7 +4103,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="24" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B27" s="28" t="n">
         <f aca="false">MIN(D26:O26)</f>
@@ -4164,7 +4112,7 @@
     </row>
     <row r="29" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -4215,7 +4163,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -4226,7 +4174,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4235,7 +4183,7 @@
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4256,7 +4204,7 @@
         <v>55</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>56</v>
@@ -4269,7 +4217,7 @@
         <v>57</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>58</v>
@@ -4368,7 +4316,7 @@
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
         <v>73</v>
       </c>
@@ -4422,7 +4370,7 @@
         <v>-800</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4440,7 +4388,7 @@
         <v>400</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,7 +4406,7 @@
         <v>-100</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4476,7 +4424,7 @@
         <v>200</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4539,7 +4487,7 @@
         <v>1500</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4557,7 +4505,7 @@
         <v>800</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4593,7 +4541,7 @@
         <v>1500</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4611,7 +4559,7 @@
         <v>300</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4629,7 +4577,7 @@
         <v>600</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4647,7 +4595,7 @@
         <v>400</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4665,7 +4613,7 @@
         <v>1200</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4683,7 +4631,7 @@
         <v>-1200</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4701,7 +4649,7 @@
         <v>700</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4719,7 +4667,7 @@
         <v/>
       </c>
       <c r="E36" s="18" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4737,7 +4685,7 @@
         <v>100</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4755,7 +4703,7 @@
         <v>900</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4773,7 +4721,7 @@
         <v>200</v>
       </c>
       <c r="E39" s="18" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4791,7 +4739,7 @@
         <v>300</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4809,7 +4757,7 @@
         <v>100</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4890,7 +4838,7 @@
         <v>6000</v>
       </c>
       <c r="E47" s="18" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4899,7 +4847,7 @@
       </c>
       <c r="C48" s="21"/>
       <c r="E48" s="21" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4948,7 +4896,7 @@
         <v>4000</v>
       </c>
       <c r="E51" s="18" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5025,11 +4973,10 @@
       <c r="E58" s="8"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="30" t="s">
+      <c r="A59" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="B59" s="31"/>
-      <c r="C59" s="32" t="n">
+      <c r="C59" s="29" t="n">
         <f aca="false">IF(OR($B$8=0,$B$9=0),"",C57/$B$8/$B$9)</f>
         <v>165.842222222222</v>
       </c>
@@ -5038,169 +4985,135 @@
       </c>
       <c r="E59" s="8"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="9" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="C60" s="29" t="n">
-        <f aca="false">IF(OR(C59="",$B$10=0),"",C59-$B$10)</f>
-        <v>5.84222222222221</v>
-      </c>
-      <c r="D60" s="8"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="32" t="n">
+        <f aca="false">IF(C59="","",C59/(1-$B$14))</f>
+        <v>174.570760233918</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>151</v>
+      </c>
       <c r="E60" s="8"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="C61" s="33" t="n">
-        <f aca="false">IF(OR(C59="",$B$10=0),"",C59/$B$10-1)</f>
-        <v>0.0365138888888887</v>
-      </c>
-      <c r="D61" s="8" t="s">
         <v>152</v>
       </c>
+      <c r="C61" s="29" t="n">
+        <f aca="false">IF(OR(C60="",$B$10=0),"",C60-$B$10)</f>
+        <v>14.5707602339181</v>
+      </c>
+      <c r="D61" s="8"/>
       <c r="E61" s="8"/>
     </row>
-    <row r="62" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="C62" s="24" t="str">
-        <f aca="false">IF(C61="","",IF($B$12="","No cap entered",IF(C61&lt;=$B$12,"Yes","Over the cap — check your documents")))</f>
-        <v>Yes</v>
+      <c r="C62" s="33" t="n">
+        <f aca="false">IF(OR(C60="",$B$10=0),"",C60/$B$10-1)</f>
+        <v>0.0910672514619884</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>154</v>
       </c>
       <c r="E62" s="8"/>
     </row>
-    <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="25" t="s">
+    <row r="63" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="B64" s="26"/>
-      <c r="C64" s="26"/>
-      <c r="D64" s="26"/>
-      <c r="E64" s="26"/>
-    </row>
-    <row r="65" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="8" t="s">
+      <c r="C63" s="24" t="str">
+        <f aca="false">IF(C62="","",IF($B$12="","No cap entered",IF(C62&lt;=$B$12,"Yes","Over the cap — check your documents")))</f>
+        <v>Yes</v>
+      </c>
+      <c r="D63" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="B65" s="8"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="8"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="34"/>
-      <c r="B66" s="35" t="s">
+      <c r="E63" s="8"/>
+    </row>
+    <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="C66" s="35" t="s">
+      <c r="B65" s="26"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="26"/>
+    </row>
+    <row r="66" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="8" t="s">
         <v>158</v>
       </c>
+      <c r="B66" s="8"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="24" t="s">
+      <c r="A67" s="34"/>
+      <c r="B67" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="B67" s="29" t="n">
-        <f aca="false">IF(C$59="","",IF($B$12="",C$59,MIN(C$59,$B$10*(1+$B$12))))</f>
-        <v>165.842222222222</v>
-      </c>
-      <c r="C67" s="17" t="n">
-        <f aca="false">IF(B67="","",(C$59-B67)*$B$8*$B$9)</f>
-        <v>0</v>
+      <c r="C67" s="35" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B68" s="29" t="n">
-        <f aca="false">IF(C$59="","",IF($B$12="",C$59,MIN(C$59,B67*(1+$B$12))))</f>
-        <v>165.842222222222</v>
+        <f aca="false">IF(C$60="","",IF($B$12="",C$60,MIN(C$60,$B$10*(1+$B$12))))</f>
+        <v>174.570760233918</v>
       </c>
       <c r="C68" s="17" t="n">
-        <f aca="false">IF(B68="","",(C$59-B68)*$B$8*$B$9)</f>
+        <f aca="false">IF(B68="","",(C$60-B68)*$B$8*$B$9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B69" s="29" t="n">
-        <f aca="false">IF(C$59="","",IF($B$12="",C$59,MIN(C$59,B68*(1+$B$12))))</f>
-        <v>165.842222222222</v>
+        <f aca="false">IF(C$60="","",IF($B$12="",C$60,MIN(C$60,B68*(1+$B$12))))</f>
+        <v>174.570760233918</v>
       </c>
       <c r="C69" s="17" t="n">
-        <f aca="false">IF(B69="","",(C$59-B69)*$B$8*$B$9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="25" t="s">
-        <v>162</v>
-      </c>
-      <c r="B71" s="26"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="26"/>
-      <c r="E71" s="26"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="9" t="s">
+        <f aca="false">IF(B69="","",(C$60-B69)*$B$8*$B$9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="C72" s="17" t="n">
-        <f aca="false">C57*$B$14</f>
-        <v>14925.8</v>
-      </c>
-      <c r="D72" s="8" t="s">
+      <c r="B70" s="29" t="n">
+        <f aca="false">IF(C$60="","",IF($B$12="",C$60,MIN(C$60,B69*(1+$B$12))))</f>
+        <v>174.570760233918</v>
+      </c>
+      <c r="C70" s="17" t="n">
+        <f aca="false">IF(B70="","",(C$60-B70)*$B$8*$B$9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="8" t="s">
         <v>164</v>
       </c>
+      <c r="B72" s="8"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="8"/>
       <c r="E72" s="8"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="C73" s="17" t="n">
-        <f aca="false">C50+$B$11</f>
-        <v>53116</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="E73" s="8"/>
-    </row>
-    <row r="74" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="C74" s="17" t="n">
-        <f aca="false">MAX(0,C72-C73)</f>
-        <v>0</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="E74" s="8"/>
-    </row>
-    <row r="76" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
     </row>
   </sheetData>
   <sheetProtection sheet="true" formatColumns="false" formatRows="false"/>
-  <mergeCells count="25">
+  <mergeCells count="23">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="C5:E5"/>
@@ -5221,11 +5134,9 @@
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="D61:E61"/>
     <mergeCell ref="D62:E62"/>
-    <mergeCell ref="A65:E65"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="D73:E73"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="A76:E76"/>
+    <mergeCell ref="D63:E63"/>
+    <mergeCell ref="A66:E66"/>
+    <mergeCell ref="A72:E72"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7" type="whole">

</xml_diff>